<commit_message>
feat: add SeasonalThemeBanner component for seasonal promotional displays
</commit_message>
<xml_diff>
--- a/data-source/banchan-50.xlsx
+++ b/data-source/banchan-50.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\K-BanChan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\K-BanChan\data-source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2EC4833-2ACD-4A30-A572-DE34DB2F57CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590DCF96-C8ED-47E4-BEAF-C4F9A3763D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="748" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="329">
   <si>
     <t>순위</t>
   </si>
@@ -1000,13 +1000,53 @@
   </si>
   <si>
     <t>X (소고기 포함)</t>
+  </si>
+  <si>
+    <t>조리법응용</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>재료 구입</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>∙</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>준비 가이드</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>비건 여부</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>반찬 스토리</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1029,6 +1069,14 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1038,7 +1086,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1061,13 +1109,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -3824,7 +3886,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="16.796875" customWidth="1"/>
@@ -3834,7 +3896,7 @@
     <col min="8" max="8" width="20.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3851,16 +3913,19 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>325</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>328</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+        <v>327</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3886,7 +3951,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>16</v>
       </c>
@@ -3912,7 +3977,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>17</v>
       </c>
@@ -3938,7 +4003,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>25</v>
       </c>
@@ -3964,7 +4029,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>27</v>
       </c>
@@ -3990,7 +4055,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>32</v>
       </c>
@@ -4016,7 +4081,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>33</v>
       </c>
@@ -4042,7 +4107,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>34</v>
       </c>
@@ -4068,7 +4133,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>40</v>
       </c>
@@ -4094,7 +4159,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>43</v>
       </c>
@@ -4120,7 +4185,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>44</v>
       </c>
@@ -4146,7 +4211,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>45</v>
       </c>
@@ -4172,7 +4237,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>47</v>
       </c>

</xml_diff>